<commit_message>
fix: remove credentials from the text of the datasets
Access tokens: where a statement linked a restricted Zenodo record
through a token, the build replaced the token's value and left the
parameter in the URL as a placeholder, so the link did not resolve. The
whole parameter is now dropped and the plain record URL kept, which is
what the helper's comment had described all along. One ploswater
article, two cells.

Stated passwords: two statements spell out a login the authors
published for their readers, an FTP site in ploswater and a file share
in ws. The password is replaced by a marker and the rest of the
sentence kept. The package does not pass credentials on.

Four cells change in total: ploswater das (2) and das_repo_url (1), ws
das (1). The gate rejects any token parameter and any stated password,
the package tests assert the same on the exported data, and the two
cleaning helpers have their own tests.

Refs #65

Assisted-by: Claude claude-fable-5-1
</commit_message>
<xml_diff>
--- a/inst/extdata/ploswater.xlsx
+++ b/inst/extdata/ploswater.xlsx
@@ -2297,10 +2297,10 @@
     <t xml:space="preserve">https://orcid.org/0000-0002-3478-2624</t>
   </si>
   <si>
-    <t xml:space="preserve">All the data used in this study are public, except the Pléiades imagery that are commercial. The Pléiades images (Pléiades © CNES 2021 Distribution AIRBUS DS) were licensed to CESBIO by Airbus. The Pléiades DEM is a derivative product subject to the CC-BY-NC 4.0 license preventing commercial use, https://creativecommons.org/licenses/by-nc/4.0/legalcode. We have publicly shared the Digital Elevation Model and derived variables on Zenodo with restricted access until the publication of the manuscript. If needed for the review, you can access to these data-sets by using these links: - 2m resolution DEM based stereoscopy Pleiades acquisitions in Telangana, South-India https://zenodo.org/records/10403040?token=[removed] - Subsample of the maximum Water Area Extent of Telangana Rainwater Harvesting System from Sentinel-2 https://zenodo.org/records/10402199?token=[removed] - Subsample of the maximum Water Area Extent of Telangana Rainwater Harvesting System from Pléiades DEM https://zenodo.org/records/10402355?token=[removed] - Maximum Water Area Extent of the Rainwater Harvesting System in Telangana from GSW https://zenodo.org/records/10402096?token=[removed]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://creativecommons.org/licenses/by-nc/4.0/legalcode; https://zenodo.org/records/10403040?token=[removed]; https://zenodo.org/records/10402199?token=[removed]; https://zenodo.org/records/10402355?token=[removed]; https://zenodo.org/records/10402096?token=[removed]</t>
+    <t xml:space="preserve">All the data used in this study are public, except the Pléiades imagery that are commercial. The Pléiades images (Pléiades © CNES 2021 Distribution AIRBUS DS) were licensed to CESBIO by Airbus. The Pléiades DEM is a derivative product subject to the CC-BY-NC 4.0 license preventing commercial use, https://creativecommons.org/licenses/by-nc/4.0/legalcode. We have publicly shared the Digital Elevation Model and derived variables on Zenodo with restricted access until the publication of the manuscript. If needed for the review, you can access to these data-sets by using these links: - 2m resolution DEM based stereoscopy Pleiades acquisitions in Telangana, South-India https://zenodo.org/records/10403040 - Subsample of the maximum Water Area Extent of Telangana Rainwater Harvesting System from Sentinel-2 https://zenodo.org/records/10402199 - Subsample of the maximum Water Area Extent of Telangana Rainwater Harvesting System from Pléiades DEM https://zenodo.org/records/10402355 - Maximum Water Area Extent of the Rainwater Harvesting System in Telangana from GSW https://zenodo.org/records/10402096</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://creativecommons.org/licenses/by-nc/4.0/legalcode; https://zenodo.org/records/10403040; https://zenodo.org/records/10402199; https://zenodo.org/records/10402355; https://zenodo.org/records/10402096</t>
   </si>
   <si>
     <t xml:space="preserve">/Biology and life sciences/Agriculture/Agricultural methods/Agricultural irrigation/Lift irrigation; /Earth sciences/Atmospheric science/Atmospheric physics/Atmospheric dynamics/Atmospheric clouds; /Earth sciences/Geophysics/Atmospheric physics/Atmospheric dynamics/Atmospheric clouds; /Earth sciences/Hydrology/Surface water; /Earth sciences/Marine and aquatic sciences/Aquatic environments/Freshwater environments/Rivers; /Earth sciences/Marine and aquatic sciences/Bodies of water/Rivers; /Ecology and environmental sciences/Aquatic environments/Freshwater environments/Rivers; /Engineering and technology/Remote sensing/Lidar; /Engineering and technology/Remote sensing/Radar; /People and places/Geographical locations/Asia/India; /Physical sciences/Physics/Geophysics/Atmospheric physics/Atmospheric dynamics/Atmospheric clouds; /Physical sciences/Physics/Particle physics/Elementary particles/Photons</t>
@@ -2555,7 +2555,7 @@
     <t xml:space="preserve">https://orcid.org/0000-0002-2165-5239</t>
   </si>
   <si>
-    <t xml:space="preserve">The JULES simulation data can be accessed at doi:10.5281/zenodo.10459886. The MERIT DEM [45] is accessible online (https://hydro.iis.utokyo. ac.jp/~yamadai/MERIT_DEM/, last access: 14 December 2023). The HESS [19,20] product is available online (https://daac.ornl.gov/LBA/guides/LC07_Amazon_Wetlands.html, last access: 15 May 2024). The GIEMS [10,40] product can be acquired by contacting Catherine Prigent ([email removed]@obspm.fr). The SWAMPS-GLWD [41] product can be acquired by contacting Zhen Zhang ([email removed]@itpcas.ac.cn). The WAD2M [43] product is available online (https://zenodo.org/records/3998454, last access: 15 May 2024). The WFDEI [48] dataset is available from the ftp site at IIASA, Vienna (ftp.iiasa.ac.at, username: rfdata password: forceDATA, then use: cwd/WFDEI, last access: 15 May 2024). The HELIX [37] data can be acquired by contacting John Ceasar ([email removed]@metoffice.gov.uk). Upon publication the JULES simulation data can be accessed at doi: 10.5281/zenodo.10459886.</t>
+    <t xml:space="preserve">The JULES simulation data can be accessed at doi:10.5281/zenodo.10459886. The MERIT DEM [45] is accessible online (https://hydro.iis.utokyo. ac.jp/~yamadai/MERIT_DEM/, last access: 14 December 2023). The HESS [19,20] product is available online (https://daac.ornl.gov/LBA/guides/LC07_Amazon_Wetlands.html, last access: 15 May 2024). The GIEMS [10,40] product can be acquired by contacting Catherine Prigent ([email removed]@obspm.fr). The SWAMPS-GLWD [41] product can be acquired by contacting Zhen Zhang ([email removed]@itpcas.ac.cn). The WAD2M [43] product is available online (https://zenodo.org/records/3998454, last access: 15 May 2024). The WFDEI [48] dataset is available from the ftp site at IIASA, Vienna (ftp.iiasa.ac.at, username: rfdata password [removed], then use: cwd/WFDEI, last access: 15 May 2024). The HELIX [37] data can be acquired by contacting John Ceasar ([email removed]@metoffice.gov.uk). Upon publication the JULES simulation data can be accessed at doi: 10.5281/zenodo.10459886.</t>
   </si>
   <si>
     <t xml:space="preserve">https://doi.org/10.5281/zenodo.10459886; https://hydro.iis.utokyo; https://daac.ornl.gov/LBA/guides/LC07_Amazon_Wetlands.html; https://zenodo.org/records/3998454; 10.5281/zenodo.10459886</t>

</xml_diff>